<commit_message>
TCs. HR1 updated to new version.
</commit_message>
<xml_diff>
--- a/data/HR1/Market Data/HR1_market_data.xlsx
+++ b/data/HR1/Market Data/HR1_market_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10817"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\thesis-shared-resources-planning-no_esso-degradation\data\CS7\Market Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/micaelsimoes/PycharmProjects/shared-resources-planning/data/HR1/Market Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{080D917E-B370-4C1E-97E4-9D9899348410}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E895503B-837A-2340-8134-6B4B52C91C63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-15195" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1060" yWindow="500" windowWidth="50140" windowHeight="28300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Growth Factors" sheetId="1" r:id="rId1"/>
@@ -388,12 +388,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -401,7 +401,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -409,7 +409,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -425,9 +425,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4C1090B-5BAB-4DF9-A5D0-788EE84E9C0B}">
   <dimension ref="A1:Z13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -507,7 +507,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -587,7 +587,7 @@
         <v>98.85560000000001</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -667,7 +667,7 @@
         <v>105.039</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -747,7 +747,7 @@
         <v>101.02120000000002</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -755,79 +755,103 @@
         <v>1</v>
       </c>
       <c r="C5" s="1">
-        <v>44</v>
+        <f>C2*(2/3)+C8*(1/3)</f>
+        <v>102.55000000000001</v>
       </c>
       <c r="D5" s="1">
-        <v>46.62</v>
+        <f t="shared" ref="D5:Z7" si="0">D2*(2/3)+D8*(1/3)</f>
+        <v>98.360533333333336</v>
       </c>
       <c r="E5" s="1">
-        <v>48.16</v>
+        <f t="shared" si="0"/>
+        <v>95.563999999999993</v>
       </c>
       <c r="F5" s="1">
-        <v>48.4</v>
+        <f t="shared" si="0"/>
+        <v>94.06</v>
       </c>
       <c r="G5" s="1">
-        <v>50.5</v>
+        <f t="shared" si="0"/>
+        <v>93.877333333333326</v>
       </c>
       <c r="H5" s="1">
-        <v>55.99</v>
+        <f t="shared" si="0"/>
+        <v>96.257333333333321</v>
       </c>
       <c r="I5" s="1">
-        <v>58.82</v>
+        <f t="shared" si="0"/>
+        <v>100.94973333333333</v>
       </c>
       <c r="J5" s="1">
-        <v>49.98</v>
+        <f t="shared" si="0"/>
+        <v>111.06199999999998</v>
       </c>
       <c r="K5" s="1">
-        <v>33.799999999999997</v>
+        <f t="shared" si="0"/>
+        <v>118.05359999999999</v>
       </c>
       <c r="L5" s="1">
-        <v>13.5</v>
+        <f t="shared" si="0"/>
+        <v>115.03999999999999</v>
       </c>
       <c r="M5" s="1">
-        <v>11.3</v>
+        <f t="shared" si="0"/>
+        <v>101.65853333333334</v>
       </c>
       <c r="N5" s="1">
-        <v>9.4499999999999993</v>
+        <f t="shared" si="0"/>
+        <v>91.893866666666668</v>
       </c>
       <c r="O5" s="1">
-        <v>4.5</v>
+        <f t="shared" si="0"/>
+        <v>90.212266666666665</v>
       </c>
       <c r="P5" s="1">
-        <v>3.13</v>
+        <f t="shared" si="0"/>
+        <v>87.737200000000001</v>
       </c>
       <c r="Q5" s="1">
-        <v>0.54</v>
+        <f t="shared" si="0"/>
+        <v>86.32</v>
       </c>
       <c r="R5" s="1">
-        <v>3.25</v>
+        <f t="shared" si="0"/>
+        <v>87.333333333333343</v>
       </c>
       <c r="S5" s="1">
-        <v>5</v>
+        <f t="shared" si="0"/>
+        <v>96.258533333333332</v>
       </c>
       <c r="T5" s="1">
-        <v>15.17</v>
+        <f t="shared" si="0"/>
+        <v>115.19666666666666</v>
       </c>
       <c r="U5" s="1">
-        <v>33.799999999999997</v>
+        <f t="shared" si="0"/>
+        <v>127.51053333333334</v>
       </c>
       <c r="V5" s="1">
-        <v>49.12</v>
+        <f t="shared" si="0"/>
+        <v>132.69906666666665</v>
       </c>
       <c r="W5" s="1">
-        <v>59.31</v>
+        <f t="shared" si="0"/>
+        <v>127.55719999999999</v>
       </c>
       <c r="X5" s="1">
-        <v>57.63</v>
+        <f t="shared" si="0"/>
+        <v>118.38653333333333</v>
       </c>
       <c r="Y5" s="1">
-        <v>49</v>
+        <f t="shared" si="0"/>
+        <v>109.71333333333332</v>
       </c>
       <c r="Z5" s="1">
-        <v>72.430000000000007</v>
-      </c>
-    </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
+        <f t="shared" si="0"/>
+        <v>103.85040000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -835,79 +859,103 @@
         <v>2</v>
       </c>
       <c r="C6" s="1">
-        <v>70.5</v>
+        <f t="shared" ref="C6:R7" si="1">C3*(2/3)+C9*(1/3)</f>
+        <v>100.992</v>
       </c>
       <c r="D6" s="1">
-        <v>69.13</v>
+        <f t="shared" si="1"/>
+        <v>99.13333333333334</v>
       </c>
       <c r="E6" s="1">
-        <v>69</v>
+        <f t="shared" si="1"/>
+        <v>98.062666666666672</v>
       </c>
       <c r="F6" s="1">
-        <v>68.010000000000005</v>
+        <f t="shared" si="1"/>
+        <v>92.533333333333331</v>
       </c>
       <c r="G6" s="1">
-        <v>68.84</v>
+        <f t="shared" si="1"/>
+        <v>95.116</v>
       </c>
       <c r="H6" s="1">
-        <v>67</v>
+        <f t="shared" si="1"/>
+        <v>97.333333333333343</v>
       </c>
       <c r="I6" s="1">
-        <v>67.92</v>
+        <f t="shared" si="1"/>
+        <v>103.63333333333333</v>
       </c>
       <c r="J6" s="1">
-        <v>72.87</v>
+        <f t="shared" si="1"/>
+        <v>107.48</v>
       </c>
       <c r="K6" s="1">
-        <v>41.7</v>
+        <f t="shared" si="1"/>
+        <v>106.15466666666666</v>
       </c>
       <c r="L6" s="1">
-        <v>30</v>
+        <f t="shared" si="1"/>
+        <v>103.46333333333334</v>
       </c>
       <c r="M6" s="1">
-        <v>18.82</v>
+        <f t="shared" si="1"/>
+        <v>99.866666666666674</v>
       </c>
       <c r="N6" s="1">
-        <v>20.43</v>
+        <f t="shared" si="1"/>
+        <v>96.391999999999996</v>
       </c>
       <c r="O6" s="1">
-        <v>14.7</v>
+        <f t="shared" si="1"/>
+        <v>94.8</v>
       </c>
       <c r="P6" s="1">
-        <v>9.66</v>
+        <f t="shared" si="1"/>
+        <v>94.801999999999992</v>
       </c>
       <c r="Q6" s="1">
-        <v>8.2100000000000009</v>
+        <f t="shared" si="1"/>
+        <v>92.606666666666655</v>
       </c>
       <c r="R6" s="1">
-        <v>7.44</v>
+        <f t="shared" si="1"/>
+        <v>94.007333333333335</v>
       </c>
       <c r="S6" s="1">
-        <v>14.7</v>
+        <f t="shared" si="0"/>
+        <v>101.38533333333334</v>
       </c>
       <c r="T6" s="1">
-        <v>19.440000000000001</v>
+        <f t="shared" si="0"/>
+        <v>106.61666666666666</v>
       </c>
       <c r="U6" s="1">
-        <v>34.79</v>
+        <f t="shared" si="0"/>
+        <v>122.06666666666666</v>
       </c>
       <c r="V6" s="1">
-        <v>62.73</v>
+        <f t="shared" si="0"/>
+        <v>126.34466666666667</v>
       </c>
       <c r="W6" s="1">
-        <v>68.010000000000005</v>
+        <f t="shared" si="0"/>
+        <v>123.63333333333334</v>
       </c>
       <c r="X6" s="1">
-        <v>66.77</v>
+        <f t="shared" si="0"/>
+        <v>115.79733333333334</v>
       </c>
       <c r="Y6" s="1">
-        <v>63.08</v>
+        <f t="shared" si="0"/>
+        <v>110.39333333333335</v>
       </c>
       <c r="Z6" s="1">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
+        <f t="shared" si="0"/>
+        <v>105.94266666666667</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -915,79 +963,103 @@
         <v>3</v>
       </c>
       <c r="C7" s="1">
-        <v>68.900000000000006</v>
+        <f t="shared" si="1"/>
+        <v>103.30646666666667</v>
       </c>
       <c r="D7" s="1">
-        <v>65.900000000000006</v>
+        <f t="shared" si="0"/>
+        <v>100.36386666666667</v>
       </c>
       <c r="E7" s="1">
-        <v>66.319999999999993</v>
+        <f t="shared" si="0"/>
+        <v>98.310600000000008</v>
       </c>
       <c r="F7" s="1">
-        <v>64.760000000000005</v>
+        <f t="shared" si="0"/>
+        <v>93.557999999999993</v>
       </c>
       <c r="G7" s="1">
-        <v>67.88</v>
+        <f t="shared" si="0"/>
+        <v>93.223333333333329</v>
       </c>
       <c r="H7" s="1">
-        <v>62.9</v>
+        <f t="shared" si="0"/>
+        <v>95.861333333333334</v>
       </c>
       <c r="I7" s="1">
-        <v>66.430000000000007</v>
+        <f t="shared" si="0"/>
+        <v>106.8</v>
       </c>
       <c r="J7" s="1">
-        <v>58.58</v>
+        <f t="shared" si="0"/>
+        <v>112.15306666666666</v>
       </c>
       <c r="K7" s="1">
-        <v>38.65</v>
+        <f t="shared" si="0"/>
+        <v>118.21733333333334</v>
       </c>
       <c r="L7" s="1">
-        <v>24.17</v>
+        <f t="shared" si="0"/>
+        <v>113.21733333333334</v>
       </c>
       <c r="M7" s="1">
-        <v>22</v>
+        <f t="shared" si="0"/>
+        <v>98.202799999999996</v>
       </c>
       <c r="N7" s="1">
-        <v>21.76</v>
+        <f t="shared" si="0"/>
+        <v>96.341533333333331</v>
       </c>
       <c r="O7" s="1">
-        <v>11.72</v>
+        <f t="shared" si="0"/>
+        <v>94.322733333333332</v>
       </c>
       <c r="P7" s="1">
-        <v>10.23</v>
+        <f t="shared" si="0"/>
+        <v>93.203333333333333</v>
       </c>
       <c r="Q7" s="1">
-        <v>3.25</v>
+        <f t="shared" si="0"/>
+        <v>89.982266666666675</v>
       </c>
       <c r="R7" s="1">
-        <v>3.25</v>
+        <f t="shared" si="0"/>
+        <v>88.837133333333341</v>
       </c>
       <c r="S7" s="1">
-        <v>8.4700000000000006</v>
+        <f t="shared" si="0"/>
+        <v>93.512199999999993</v>
       </c>
       <c r="T7" s="1">
-        <v>25.1</v>
+        <f t="shared" si="0"/>
+        <v>97.958666666666673</v>
       </c>
       <c r="U7" s="1">
-        <v>41.2</v>
+        <f t="shared" si="0"/>
+        <v>109.38073333333332</v>
       </c>
       <c r="V7" s="1">
-        <v>57.24</v>
+        <f t="shared" si="0"/>
+        <v>124.55733333333333</v>
       </c>
       <c r="W7" s="1">
-        <v>74.63</v>
+        <f t="shared" si="0"/>
+        <v>125.28666666666666</v>
       </c>
       <c r="X7" s="1">
-        <v>67.88</v>
+        <f t="shared" si="0"/>
+        <v>114.44926666666666</v>
       </c>
       <c r="Y7" s="1">
-        <v>71</v>
+        <f t="shared" si="0"/>
+        <v>105.0192</v>
       </c>
       <c r="Z7" s="1">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
+        <f t="shared" si="0"/>
+        <v>92.090800000000002</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -1067,7 +1139,7 @@
         <v>113.84</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -1147,7 +1219,7 @@
         <v>107.75</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>7</v>
       </c>
@@ -1227,7 +1299,7 @@
         <v>74.23</v>
       </c>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -1307,7 +1379,7 @@
         <v>109.64</v>
       </c>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -1387,7 +1459,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -1475,9 +1547,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45EAE8BD-6C17-44DF-B187-38D65FB995D2}">
   <dimension ref="A1:Z13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -1557,7 +1629,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1637,7 +1709,7 @@
         <v>65.306785500000004</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -1717,7 +1789,7 @@
         <v>59.761869749999995</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -1797,7 +1869,7 @@
         <v>65.256999500000006</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -1877,7 +1949,7 @@
         <v>63.3909375</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -1957,7 +2029,7 @@
         <v>63.3909375</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -2037,7 +2109,7 @@
         <v>62.750624999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -2117,7 +2189,7 @@
         <v>72.373199999999997</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -2197,7 +2269,7 @@
         <v>76.142637500000006</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>7</v>
       </c>
@@ -2277,7 +2349,7 @@
         <v>79.158187499999997</v>
       </c>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -2357,7 +2429,7 @@
         <v>74.325900000000004</v>
       </c>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -2437,7 +2509,7 @@
         <v>73.59</v>
       </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>8</v>
       </c>

</xml_diff>